<commit_message>
estadisticas descriptivas y regresiones finales
</commit_message>
<xml_diff>
--- a/src/codigo/reviewers/results/salario.xlsx
+++ b/src/codigo/reviewers/results/salario.xlsx
@@ -19,16 +19,16 @@
     <t>logro</t>
   </si>
   <si>
-    <t>w_promedio_Costa Rica</t>
-  </si>
-  <si>
-    <t>w_promedio_Nicaragua</t>
-  </si>
-  <si>
-    <t>N_Costa Rica</t>
-  </si>
-  <si>
-    <t>N_Nicaragua</t>
+    <t>w_promedio_nicaraguense</t>
+  </si>
+  <si>
+    <t>w_promedio_costarricense</t>
+  </si>
+  <si>
+    <t>N_nicaraguense</t>
+  </si>
+  <si>
+    <t>N_costarricense</t>
   </si>
   <si>
     <t>Primaria Incompleta</t>
@@ -109,10 +109,10 @@
   <autoFilter ref="A1:E6"/>
   <tableColumns count="5">
     <tableColumn id="1" name="logro" dataDxfId="0"/>
-    <tableColumn id="2" name="w_promedio_Costa Rica" dataDxfId="1"/>
-    <tableColumn id="3" name="w_promedio_Nicaragua" dataDxfId="1"/>
-    <tableColumn id="4" name="N_Costa Rica" dataDxfId="1"/>
-    <tableColumn id="5" name="N_Nicaragua" dataDxfId="1"/>
+    <tableColumn id="2" name="w_promedio_nicaraguense" dataDxfId="1"/>
+    <tableColumn id="3" name="w_promedio_costarricense" dataDxfId="1"/>
+    <tableColumn id="4" name="N_nicaraguense" dataDxfId="1"/>
+    <tableColumn id="5" name="N_costarricense" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -428,16 +428,16 @@
         <v>5</v>
       </c>
       <c r="B2" s="2">
-        <v>1436.41</v>
+        <v>1991.69</v>
       </c>
       <c r="C2" s="2">
-        <v>1553.97</v>
+        <v>1756.44</v>
       </c>
       <c r="D2" s="2">
-        <v>142850</v>
+        <v>15094</v>
       </c>
       <c r="E2" s="2">
-        <v>82601</v>
+        <v>23118</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -445,16 +445,16 @@
         <v>6</v>
       </c>
       <c r="B3" s="2">
-        <v>1559.09</v>
+        <v>2577.78</v>
       </c>
       <c r="C3" s="2">
-        <v>1653.79</v>
+        <v>2045</v>
       </c>
       <c r="D3" s="2">
-        <v>598883</v>
+        <v>21893</v>
       </c>
       <c r="E3" s="2">
-        <v>97770</v>
+        <v>86213</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -462,16 +462,16 @@
         <v>7</v>
       </c>
       <c r="B4" s="2">
-        <v>1691.18</v>
+        <v>1978.8</v>
       </c>
       <c r="C4" s="2">
-        <v>1623.4</v>
+        <v>2160.26</v>
       </c>
       <c r="D4" s="2">
-        <v>659698</v>
+        <v>15518</v>
       </c>
       <c r="E4" s="2">
-        <v>118299</v>
+        <v>76235</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -479,16 +479,16 @@
         <v>8</v>
       </c>
       <c r="B5" s="2">
-        <v>2083.43</v>
+        <v>2174.11</v>
       </c>
       <c r="C5" s="2">
-        <v>1741.82</v>
+        <v>2587.16</v>
       </c>
       <c r="D5" s="2">
-        <v>626665</v>
+        <v>13920</v>
       </c>
       <c r="E5" s="2">
-        <v>71211</v>
+        <v>156144</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -496,16 +496,16 @@
         <v>9</v>
       </c>
       <c r="B6" s="2">
-        <v>4958.4</v>
+        <v>4496.57</v>
       </c>
       <c r="C6" s="2">
-        <v>3104.12</v>
+        <v>5767.78</v>
       </c>
       <c r="D6" s="2">
-        <v>1465609</v>
+        <v>6678</v>
       </c>
       <c r="E6" s="2">
-        <v>38023</v>
+        <v>282499</v>
       </c>
     </row>
   </sheetData>

</xml_diff>